<commit_message>
added docker, fastapi notes
</commit_message>
<xml_diff>
--- a/AI/Core_GenAI_AgenticAI_Topic_Map.xlsx
+++ b/AI/Core_GenAI_AgenticAI_Topic_Map.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\REHAN ASHRAF\OneDrive\Desktop\learning\AI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d5c410d65fba7c6e/Desktop/learning/AI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5B0FDB-B315-4E46-891F-B37800A4DF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{EE5B0FDB-B315-4E46-891F-B37800A4DF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C733F809-97C1-443C-A057-9DE8D563126F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -909,10 +909,6 @@
 • ToolMessage</t>
   </si>
   <si>
-    <t>• add_messages
-• MessagesState</t>
-  </si>
-  <si>
     <t>• Responses API messages
 • Threads/messages in Azure AI Agents</t>
   </si>
@@ -1348,6 +1344,11 @@
 • Tool execution
 • Tool error handling 
 • MCP</t>
+  </si>
+  <si>
+    <t>• add_messages
+• MessagesState
+• AgentState</t>
   </si>
 </sst>
 </file>
@@ -1830,10 +1831,10 @@
         <v>168</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="64" customHeight="1">
@@ -1841,16 +1842,16 @@
         <v>75</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="64" customHeight="1">
@@ -1858,84 +1859,84 @@
         <v>80</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="64" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="64" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="64" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="64" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>197</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2197,7 +2198,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="83" customHeight="1">
+    <row r="8" spans="1:5" ht="93" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>75</v>
       </c>
@@ -2361,7 +2362,7 @@
         <v>111</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>112</v>
@@ -2389,7 +2390,7 @@
     </row>
     <row r="4" spans="1:5" ht="68.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>119</v>
@@ -2426,7 +2427,7 @@
         <v>128</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>129</v>
@@ -2477,7 +2478,7 @@
         <v>142</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>143</v>
@@ -2544,22 +2545,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1">
       <c r="A1" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>203</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="64" customHeight="1">
@@ -2567,19 +2568,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>208</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="64" customHeight="1">
@@ -2587,19 +2588,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>213</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="64" customHeight="1">
@@ -2607,19 +2608,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>217</v>
-      </c>
       <c r="F4" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="64" customHeight="1">
@@ -2627,19 +2628,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>221</v>
-      </c>
       <c r="F5" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="64" customHeight="1">
@@ -2647,19 +2648,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>225</v>
-      </c>
       <c r="F6" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2691,209 +2692,209 @@
         <v>156</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28" customHeight="1">
       <c r="A2" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>231</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28" customHeight="1">
       <c r="A3" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>235</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>243</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="28" customHeight="1">
       <c r="A6" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>247</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28" customHeight="1">
       <c r="A7" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>251</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="28" customHeight="1">
       <c r="A8" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>255</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28" customHeight="1">
       <c r="A9" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>259</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>263</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>267</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="28" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>270</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="28" customHeight="1">
       <c r="A13" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>274</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28" customHeight="1">
       <c r="A14" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>278</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="28" customHeight="1">
       <c r="A15" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>281</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>282</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>